<commit_message>
Update on 4.30 New Product Image 2
</commit_message>
<xml_diff>
--- a/resources/4.30 新增产品.xlsx
+++ b/resources/4.30 新增产品.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hengchangqi/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hengchangqi/Documents/Singapore/Plan &amp; Note Internship/Part Time/WeChatProjects/TrinityGlobe/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{99EC31E4-78FE-1147-9D80-5100EEAC6C11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DB8513C-EEDB-6B47-8D53-B91AE5953F79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -295,6 +295,7 @@
     <font>
       <sz val="12"/>
       <name val="Microsoft YaHei"/>
+      <family val="2"/>
       <charset val="134"/>
     </font>
     <font>
@@ -304,7 +305,7 @@
       <charset val="134"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -341,6 +342,12 @@
         <bgColor auto="1"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -356,7 +363,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -375,25 +382,31 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -660,7 +673,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="18" customHeight="1">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="7"/>
@@ -700,10 +713,10 @@
       <c r="X1" s="2"/>
     </row>
     <row r="2" spans="1:24" ht="18" customHeight="1">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="7"/>
+      <c r="B2" s="13"/>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
@@ -728,10 +741,10 @@
       <c r="X2" s="2"/>
     </row>
     <row r="3" spans="1:24" ht="18" customHeight="1">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="7"/>
+      <c r="B3" s="13"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2">
         <v>131</v>
@@ -760,10 +773,10 @@
       <c r="X3" s="2"/>
     </row>
     <row r="4" spans="1:24" ht="18" customHeight="1">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="7"/>
+      <c r="B4" s="13"/>
       <c r="C4" s="2"/>
       <c r="D4" s="2">
         <v>147</v>
@@ -792,10 +805,10 @@
       <c r="X4" s="2"/>
     </row>
     <row r="5" spans="1:24" ht="18" customHeight="1">
-      <c r="A5" s="9" t="s">
+      <c r="A5" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="7"/>
+      <c r="B5" s="13"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2">
         <v>240</v>
@@ -824,10 +837,10 @@
       <c r="X5" s="2"/>
     </row>
     <row r="6" spans="1:24" ht="18" customHeight="1">
-      <c r="A6" s="9" t="s">
+      <c r="A6" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="7"/>
+      <c r="B6" s="13"/>
       <c r="C6" s="2"/>
       <c r="D6" s="2">
         <v>448</v>
@@ -856,10 +869,10 @@
       <c r="X6" s="2"/>
     </row>
     <row r="7" spans="1:24" ht="18" customHeight="1">
-      <c r="A7" s="9" t="s">
+      <c r="A7" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="7"/>
+      <c r="B7" s="13"/>
       <c r="C7" s="2"/>
       <c r="D7" s="2">
         <v>540</v>
@@ -888,10 +901,10 @@
       <c r="X7" s="2"/>
     </row>
     <row r="8" spans="1:24" ht="18" customHeight="1">
-      <c r="A8" s="9" t="s">
+      <c r="A8" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="7"/>
+      <c r="B8" s="13"/>
       <c r="C8" s="2"/>
       <c r="D8" s="2">
         <v>2800</v>
@@ -920,10 +933,10 @@
       <c r="X8" s="2"/>
     </row>
     <row r="9" spans="1:24" ht="18" customHeight="1">
-      <c r="A9" s="9" t="s">
+      <c r="A9" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="7"/>
+      <c r="B9" s="13"/>
       <c r="C9" s="2"/>
       <c r="D9" s="2">
         <v>4690</v>
@@ -952,10 +965,10 @@
       <c r="X9" s="2"/>
     </row>
     <row r="10" spans="1:24" ht="18" customHeight="1">
-      <c r="A10" s="9" t="s">
+      <c r="A10" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="7"/>
+      <c r="B10" s="13"/>
       <c r="C10" s="2"/>
       <c r="D10" s="2">
         <v>6800</v>
@@ -984,7 +997,7 @@
       <c r="X10" s="2"/>
     </row>
     <row r="11" spans="1:24" ht="18" customHeight="1">
-      <c r="A11" s="8" t="s">
+      <c r="A11" s="10" t="s">
         <v>16</v>
       </c>
       <c r="B11" s="7"/>
@@ -1012,10 +1025,10 @@
       <c r="X11" s="2"/>
     </row>
     <row r="12" spans="1:24" ht="18" customHeight="1">
-      <c r="A12" s="9" t="s">
+      <c r="A12" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="7"/>
+      <c r="B12" s="13"/>
       <c r="C12" s="2">
         <v>129</v>
       </c>
@@ -1046,10 +1059,10 @@
       <c r="X12" s="2"/>
     </row>
     <row r="13" spans="1:24" ht="18" customHeight="1">
-      <c r="A13" s="9" t="s">
+      <c r="A13" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="B13" s="7"/>
+      <c r="B13" s="13"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2">
         <v>858</v>
@@ -1078,10 +1091,10 @@
       <c r="X13" s="2"/>
     </row>
     <row r="14" spans="1:24" ht="18" customHeight="1">
-      <c r="A14" s="9" t="s">
+      <c r="A14" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B14" s="7"/>
+      <c r="B14" s="13"/>
       <c r="C14" s="2">
         <v>237</v>
       </c>
@@ -1112,10 +1125,10 @@
       <c r="X14" s="2"/>
     </row>
     <row r="15" spans="1:24" ht="18" customHeight="1">
-      <c r="A15" s="9" t="s">
+      <c r="A15" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="B15" s="7"/>
+      <c r="B15" s="13"/>
       <c r="C15" s="2"/>
       <c r="D15" s="2">
         <v>1038</v>
@@ -1144,7 +1157,7 @@
       <c r="X15" s="2"/>
     </row>
     <row r="16" spans="1:24" ht="18" customHeight="1">
-      <c r="A16" s="8" t="s">
+      <c r="A16" s="10" t="s">
         <v>21</v>
       </c>
       <c r="B16" s="7"/>
@@ -1172,10 +1185,10 @@
       <c r="X16" s="2"/>
     </row>
     <row r="17" spans="1:24" ht="18" customHeight="1">
-      <c r="A17" s="9" t="s">
+      <c r="A17" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B17" s="7"/>
+      <c r="B17" s="13"/>
       <c r="C17" s="2"/>
       <c r="D17" s="2">
         <v>89</v>
@@ -1204,10 +1217,10 @@
       <c r="X17" s="2"/>
     </row>
     <row r="18" spans="1:24" ht="18" customHeight="1">
-      <c r="A18" s="9" t="s">
+      <c r="A18" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="B18" s="7"/>
+      <c r="B18" s="13"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2">
         <v>232</v>
@@ -1236,10 +1249,10 @@
       <c r="X18" s="2"/>
     </row>
     <row r="19" spans="1:24" ht="18" customHeight="1">
-      <c r="A19" s="9" t="s">
+      <c r="A19" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="B19" s="7"/>
+      <c r="B19" s="13"/>
       <c r="C19" s="2"/>
       <c r="D19" s="2">
         <v>1398</v>
@@ -1268,10 +1281,10 @@
       <c r="X19" s="2"/>
     </row>
     <row r="20" spans="1:24" ht="18" customHeight="1">
-      <c r="A20" s="9" t="s">
+      <c r="A20" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="B20" s="7"/>
+      <c r="B20" s="13"/>
       <c r="C20" s="2">
         <v>77</v>
       </c>
@@ -1302,10 +1315,10 @@
       <c r="X20" s="2"/>
     </row>
     <row r="21" spans="1:24" ht="18" customHeight="1">
-      <c r="A21" s="9" t="s">
+      <c r="A21" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="B21" s="7"/>
+      <c r="B21" s="13"/>
       <c r="C21" s="2">
         <v>200</v>
       </c>
@@ -1336,10 +1349,10 @@
       <c r="X21" s="2"/>
     </row>
     <row r="22" spans="1:24" ht="18" customHeight="1">
-      <c r="A22" s="10" t="s">
+      <c r="A22" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="B22" s="7"/>
+      <c r="B22" s="13"/>
       <c r="C22" s="5"/>
       <c r="D22" s="5"/>
       <c r="E22" s="5">
@@ -1366,10 +1379,10 @@
       <c r="X22" s="2"/>
     </row>
     <row r="23" spans="1:24" ht="18" customHeight="1">
-      <c r="A23" s="10" t="s">
+      <c r="A23" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="B23" s="7"/>
+      <c r="B23" s="13"/>
       <c r="C23" s="5"/>
       <c r="D23" s="5"/>
       <c r="E23" s="5">
@@ -1396,7 +1409,7 @@
       <c r="X23" s="2"/>
     </row>
     <row r="24" spans="1:24" ht="18" customHeight="1">
-      <c r="A24" s="8" t="s">
+      <c r="A24" s="10" t="s">
         <v>29</v>
       </c>
       <c r="B24" s="7"/>
@@ -1424,10 +1437,10 @@
       <c r="X24" s="2"/>
     </row>
     <row r="25" spans="1:24" ht="18" customHeight="1">
-      <c r="A25" s="9" t="s">
+      <c r="A25" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="B25" s="7"/>
+      <c r="B25" s="13"/>
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
       <c r="E25" s="2">
@@ -1454,10 +1467,10 @@
       <c r="X25" s="2"/>
     </row>
     <row r="26" spans="1:24" ht="18" customHeight="1">
-      <c r="A26" s="9" t="s">
+      <c r="A26" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="B26" s="7"/>
+      <c r="B26" s="13"/>
       <c r="C26" s="2"/>
       <c r="D26" s="2"/>
       <c r="E26" s="2">
@@ -1484,10 +1497,10 @@
       <c r="X26" s="2"/>
     </row>
     <row r="27" spans="1:24" ht="18" customHeight="1">
-      <c r="A27" s="9" t="s">
+      <c r="A27" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="B27" s="7"/>
+      <c r="B27" s="13"/>
       <c r="C27" s="2"/>
       <c r="D27" s="2"/>
       <c r="E27" s="2">
@@ -1514,10 +1527,10 @@
       <c r="X27" s="2"/>
     </row>
     <row r="28" spans="1:24" ht="18" customHeight="1">
-      <c r="A28" s="9" t="s">
+      <c r="A28" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="B28" s="7"/>
+      <c r="B28" s="13"/>
       <c r="C28" s="2"/>
       <c r="D28" s="2"/>
       <c r="E28" s="2">
@@ -1544,10 +1557,10 @@
       <c r="X28" s="2"/>
     </row>
     <row r="29" spans="1:24" ht="18" customHeight="1">
-      <c r="A29" s="9" t="s">
+      <c r="A29" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="B29" s="7"/>
+      <c r="B29" s="13"/>
       <c r="C29" s="2"/>
       <c r="D29" s="2"/>
       <c r="E29" s="2">
@@ -1574,10 +1587,10 @@
       <c r="X29" s="2"/>
     </row>
     <row r="30" spans="1:24" ht="18" customHeight="1">
-      <c r="A30" s="9" t="s">
+      <c r="A30" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="B30" s="7"/>
+      <c r="B30" s="13"/>
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
       <c r="E30" s="2">
@@ -1604,10 +1617,10 @@
       <c r="X30" s="2"/>
     </row>
     <row r="31" spans="1:24" ht="18" customHeight="1">
-      <c r="A31" s="9" t="s">
+      <c r="A31" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="B31" s="7"/>
+      <c r="B31" s="13"/>
       <c r="C31" s="2"/>
       <c r="D31" s="2"/>
       <c r="E31" s="2">
@@ -1634,10 +1647,10 @@
       <c r="X31" s="2"/>
     </row>
     <row r="32" spans="1:24" ht="18" customHeight="1">
-      <c r="A32" s="9" t="s">
+      <c r="A32" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="B32" s="7"/>
+      <c r="B32" s="13"/>
       <c r="C32" s="2"/>
       <c r="D32" s="2"/>
       <c r="E32" s="2">
@@ -1664,10 +1677,10 @@
       <c r="X32" s="2"/>
     </row>
     <row r="33" spans="1:24" ht="18" customHeight="1">
-      <c r="A33" s="9" t="s">
+      <c r="A33" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="B33" s="7"/>
+      <c r="B33" s="13"/>
       <c r="C33" s="2"/>
       <c r="D33" s="2"/>
       <c r="E33" s="2">
@@ -1694,10 +1707,10 @@
       <c r="X33" s="2"/>
     </row>
     <row r="34" spans="1:24" ht="18" customHeight="1">
-      <c r="A34" s="9" t="s">
+      <c r="A34" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="B34" s="7"/>
+      <c r="B34" s="13"/>
       <c r="C34" s="2"/>
       <c r="D34" s="2"/>
       <c r="E34" s="2">
@@ -1724,10 +1737,10 @@
       <c r="X34" s="2"/>
     </row>
     <row r="35" spans="1:24" ht="18" customHeight="1">
-      <c r="A35" s="9" t="s">
+      <c r="A35" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="B35" s="7"/>
+      <c r="B35" s="13"/>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
       <c r="E35" s="2">
@@ -1754,10 +1767,10 @@
       <c r="X35" s="2"/>
     </row>
     <row r="36" spans="1:24" ht="18" customHeight="1">
-      <c r="A36" s="9" t="s">
+      <c r="A36" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="B36" s="7"/>
+      <c r="B36" s="13"/>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
       <c r="E36" s="2">
@@ -1784,10 +1797,10 @@
       <c r="X36" s="2"/>
     </row>
     <row r="37" spans="1:24" ht="18" customHeight="1">
-      <c r="A37" s="9" t="s">
+      <c r="A37" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="B37" s="7"/>
+      <c r="B37" s="13"/>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>
       <c r="E37" s="2">
@@ -1814,7 +1827,7 @@
       <c r="X37" s="2"/>
     </row>
     <row r="38" spans="1:24" ht="18" customHeight="1">
-      <c r="A38" s="8" t="s">
+      <c r="A38" s="10" t="s">
         <v>43</v>
       </c>
       <c r="B38" s="7"/>
@@ -1842,10 +1855,10 @@
       <c r="X38" s="2"/>
     </row>
     <row r="39" spans="1:24" ht="18" customHeight="1">
-      <c r="A39" s="9" t="s">
+      <c r="A39" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="B39" s="7"/>
+      <c r="B39" s="13"/>
       <c r="C39" s="2"/>
       <c r="D39" s="2"/>
       <c r="E39" s="2">
@@ -1872,10 +1885,10 @@
       <c r="X39" s="2"/>
     </row>
     <row r="40" spans="1:24" ht="18" customHeight="1">
-      <c r="A40" s="9" t="s">
+      <c r="A40" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="B40" s="7"/>
+      <c r="B40" s="13"/>
       <c r="C40" s="2"/>
       <c r="D40" s="2"/>
       <c r="E40" s="2">
@@ -1902,7 +1915,7 @@
       <c r="X40" s="2"/>
     </row>
     <row r="41" spans="1:24" ht="18" customHeight="1">
-      <c r="A41" s="9" t="s">
+      <c r="A41" s="6" t="s">
         <v>46</v>
       </c>
       <c r="B41" s="7"/>
@@ -1932,7 +1945,7 @@
       <c r="X41" s="2"/>
     </row>
     <row r="42" spans="1:24" ht="18" customHeight="1">
-      <c r="A42" s="9" t="s">
+      <c r="A42" s="6" t="s">
         <v>47</v>
       </c>
       <c r="B42" s="7"/>
@@ -1962,7 +1975,7 @@
       <c r="X42" s="2"/>
     </row>
     <row r="43" spans="1:24" ht="18" customHeight="1">
-      <c r="A43" s="9" t="s">
+      <c r="A43" s="6" t="s">
         <v>48</v>
       </c>
       <c r="B43" s="7"/>
@@ -1992,7 +2005,7 @@
       <c r="X43" s="2"/>
     </row>
     <row r="44" spans="1:24">
-      <c r="A44" s="9" t="s">
+      <c r="A44" s="6" t="s">
         <v>49</v>
       </c>
       <c r="B44" s="7"/>
@@ -2022,10 +2035,10 @@
       <c r="X44" s="2"/>
     </row>
     <row r="45" spans="1:24">
-      <c r="A45" s="9" t="s">
+      <c r="A45" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="B45" s="7"/>
+      <c r="B45" s="13"/>
       <c r="C45" s="2"/>
       <c r="D45" s="2"/>
       <c r="E45" s="2">
@@ -2052,10 +2065,10 @@
       <c r="X45" s="2"/>
     </row>
     <row r="46" spans="1:24">
-      <c r="A46" s="9" t="s">
+      <c r="A46" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="B46" s="7"/>
+      <c r="B46" s="13"/>
       <c r="C46" s="2"/>
       <c r="D46" s="2"/>
       <c r="E46" s="2">
@@ -2082,10 +2095,10 @@
       <c r="X46" s="2"/>
     </row>
     <row r="47" spans="1:24">
-      <c r="A47" s="9" t="s">
+      <c r="A47" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="B47" s="7"/>
+      <c r="B47" s="13"/>
       <c r="C47" s="2"/>
       <c r="D47" s="2"/>
       <c r="E47" s="2">
@@ -2112,10 +2125,10 @@
       <c r="X47" s="2"/>
     </row>
     <row r="48" spans="1:24">
-      <c r="A48" s="9" t="s">
+      <c r="A48" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="B48" s="7"/>
+      <c r="B48" s="13"/>
       <c r="C48" s="2"/>
       <c r="D48" s="2"/>
       <c r="E48" s="2">
@@ -2142,10 +2155,10 @@
       <c r="X48" s="2"/>
     </row>
     <row r="49" spans="1:24">
-      <c r="A49" s="9" t="s">
+      <c r="A49" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="B49" s="7"/>
+      <c r="B49" s="13"/>
       <c r="C49" s="2"/>
       <c r="D49" s="2"/>
       <c r="E49" s="2">
@@ -2172,10 +2185,10 @@
       <c r="X49" s="2"/>
     </row>
     <row r="50" spans="1:24">
-      <c r="A50" s="9" t="s">
+      <c r="A50" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="B50" s="7"/>
+      <c r="B50" s="13"/>
       <c r="C50" s="2"/>
       <c r="D50" s="2"/>
       <c r="E50" s="2">
@@ -2202,10 +2215,10 @@
       <c r="X50" s="2"/>
     </row>
     <row r="51" spans="1:24">
-      <c r="A51" s="9" t="s">
+      <c r="A51" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="B51" s="7"/>
+      <c r="B51" s="13"/>
       <c r="C51" s="2"/>
       <c r="D51" s="2"/>
       <c r="E51" s="2">
@@ -2232,10 +2245,10 @@
       <c r="X51" s="2"/>
     </row>
     <row r="52" spans="1:24">
-      <c r="A52" s="9" t="s">
+      <c r="A52" s="12" t="s">
         <v>57</v>
       </c>
-      <c r="B52" s="7"/>
+      <c r="B52" s="13"/>
       <c r="C52" s="2"/>
       <c r="D52" s="2"/>
       <c r="E52" s="2">
@@ -2262,7 +2275,7 @@
       <c r="X52" s="2"/>
     </row>
     <row r="53" spans="1:24">
-      <c r="A53" s="8" t="s">
+      <c r="A53" s="10" t="s">
         <v>58</v>
       </c>
       <c r="B53" s="7"/>
@@ -2290,10 +2303,10 @@
       <c r="X53" s="2"/>
     </row>
     <row r="54" spans="1:24">
-      <c r="A54" s="9" t="s">
+      <c r="A54" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="B54" s="7"/>
+      <c r="B54" s="13"/>
       <c r="C54" s="2"/>
       <c r="D54" s="2"/>
       <c r="E54" s="2">
@@ -2320,10 +2333,10 @@
       <c r="X54" s="2"/>
     </row>
     <row r="55" spans="1:24">
-      <c r="A55" s="9" t="s">
+      <c r="A55" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="B55" s="7"/>
+      <c r="B55" s="13"/>
       <c r="C55" s="2"/>
       <c r="D55" s="2"/>
       <c r="E55" s="2">
@@ -2350,10 +2363,10 @@
       <c r="X55" s="2"/>
     </row>
     <row r="56" spans="1:24">
-      <c r="A56" s="9" t="s">
+      <c r="A56" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="B56" s="7"/>
+      <c r="B56" s="13"/>
       <c r="C56" s="2"/>
       <c r="D56" s="2"/>
       <c r="E56" s="2">
@@ -2380,10 +2393,10 @@
       <c r="X56" s="2"/>
     </row>
     <row r="57" spans="1:24">
-      <c r="A57" s="9" t="s">
+      <c r="A57" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="B57" s="7"/>
+      <c r="B57" s="13"/>
       <c r="C57" s="2"/>
       <c r="D57" s="2"/>
       <c r="E57" s="2">
@@ -2410,10 +2423,10 @@
       <c r="X57" s="2"/>
     </row>
     <row r="58" spans="1:24">
-      <c r="A58" s="9" t="s">
+      <c r="A58" s="12" t="s">
         <v>63</v>
       </c>
-      <c r="B58" s="7"/>
+      <c r="B58" s="13"/>
       <c r="C58" s="2"/>
       <c r="D58" s="2">
         <v>228</v>
@@ -2442,10 +2455,10 @@
       <c r="X58" s="2"/>
     </row>
     <row r="59" spans="1:24">
-      <c r="A59" s="9" t="s">
+      <c r="A59" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="B59" s="7"/>
+      <c r="B59" s="13"/>
       <c r="C59" s="2"/>
       <c r="D59" s="2">
         <v>340</v>
@@ -2474,10 +2487,10 @@
       <c r="X59" s="2"/>
     </row>
     <row r="60" spans="1:24">
-      <c r="A60" s="9" t="s">
+      <c r="A60" s="12" t="s">
         <v>65</v>
       </c>
-      <c r="B60" s="7"/>
+      <c r="B60" s="13"/>
       <c r="C60" s="2"/>
       <c r="D60" s="2"/>
       <c r="E60" s="4">
@@ -2504,10 +2517,10 @@
       <c r="X60" s="2"/>
     </row>
     <row r="61" spans="1:24">
-      <c r="A61" s="9" t="s">
+      <c r="A61" s="12" t="s">
         <v>66</v>
       </c>
-      <c r="B61" s="7"/>
+      <c r="B61" s="13"/>
       <c r="C61" s="2"/>
       <c r="D61" s="2"/>
       <c r="E61" s="4">
@@ -2534,10 +2547,10 @@
       <c r="X61" s="2"/>
     </row>
     <row r="62" spans="1:24">
-      <c r="A62" s="9" t="s">
+      <c r="A62" s="12" t="s">
         <v>67</v>
       </c>
-      <c r="B62" s="7"/>
+      <c r="B62" s="13"/>
       <c r="C62" s="2"/>
       <c r="D62" s="2"/>
       <c r="E62" s="4">
@@ -2564,10 +2577,10 @@
       <c r="X62" s="2"/>
     </row>
     <row r="63" spans="1:24">
-      <c r="A63" s="9" t="s">
+      <c r="A63" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="B63" s="7"/>
+      <c r="B63" s="13"/>
       <c r="C63" s="2"/>
       <c r="D63" s="2"/>
       <c r="E63" s="4">
@@ -2594,7 +2607,7 @@
       <c r="X63" s="2"/>
     </row>
     <row r="64" spans="1:24">
-      <c r="A64" s="8" t="s">
+      <c r="A64" s="10" t="s">
         <v>69</v>
       </c>
       <c r="B64" s="7"/>
@@ -2622,10 +2635,10 @@
       <c r="X64" s="2"/>
     </row>
     <row r="65" spans="1:24">
-      <c r="A65" s="9" t="s">
+      <c r="A65" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="B65" s="7"/>
+      <c r="B65" s="13"/>
       <c r="C65" s="2"/>
       <c r="D65" s="2">
         <v>324</v>
@@ -2654,10 +2667,10 @@
       <c r="X65" s="2"/>
     </row>
     <row r="66" spans="1:24">
-      <c r="A66" s="9" t="s">
+      <c r="A66" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="B66" s="7"/>
+      <c r="B66" s="13"/>
       <c r="C66" s="2"/>
       <c r="D66" s="2">
         <v>263</v>
@@ -2686,10 +2699,10 @@
       <c r="X66" s="2"/>
     </row>
     <row r="67" spans="1:24">
-      <c r="A67" s="9" t="s">
+      <c r="A67" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="B67" s="7"/>
+      <c r="B67" s="13"/>
       <c r="C67" s="2"/>
       <c r="D67" s="2">
         <v>496</v>
@@ -2718,10 +2731,10 @@
       <c r="X67" s="2"/>
     </row>
     <row r="68" spans="1:24">
-      <c r="A68" s="9" t="s">
+      <c r="A68" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="B68" s="7"/>
+      <c r="B68" s="13"/>
       <c r="C68" s="2"/>
       <c r="D68" s="2">
         <v>88</v>
@@ -2750,10 +2763,10 @@
       <c r="X68" s="2"/>
     </row>
     <row r="69" spans="1:24">
-      <c r="A69" s="9" t="s">
+      <c r="A69" s="12" t="s">
         <v>74</v>
       </c>
-      <c r="B69" s="7"/>
+      <c r="B69" s="13"/>
       <c r="C69" s="2"/>
       <c r="D69" s="2">
         <v>116</v>
@@ -2782,10 +2795,10 @@
       <c r="X69" s="2"/>
     </row>
     <row r="70" spans="1:24">
-      <c r="A70" s="9" t="s">
+      <c r="A70" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="B70" s="7"/>
+      <c r="B70" s="13"/>
       <c r="C70" s="2"/>
       <c r="D70" s="2">
         <v>124</v>
@@ -2814,10 +2827,10 @@
       <c r="X70" s="2"/>
     </row>
     <row r="71" spans="1:24">
-      <c r="A71" s="10" t="s">
+      <c r="A71" s="12" t="s">
         <v>76</v>
       </c>
-      <c r="B71" s="7"/>
+      <c r="B71" s="13"/>
       <c r="C71" s="5"/>
       <c r="D71" s="5"/>
       <c r="E71" s="5">
@@ -2844,10 +2857,10 @@
       <c r="X71" s="2"/>
     </row>
     <row r="72" spans="1:24">
-      <c r="A72" s="10" t="s">
+      <c r="A72" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="B72" s="7"/>
+      <c r="B72" s="13"/>
       <c r="C72" s="5"/>
       <c r="D72" s="5"/>
       <c r="E72" s="5">
@@ -2874,10 +2887,10 @@
       <c r="X72" s="2"/>
     </row>
     <row r="73" spans="1:24">
-      <c r="A73" s="10" t="s">
+      <c r="A73" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="B73" s="7"/>
+      <c r="B73" s="13"/>
       <c r="C73" s="5"/>
       <c r="D73" s="5"/>
       <c r="E73" s="5">
@@ -2904,10 +2917,10 @@
       <c r="X73" s="2"/>
     </row>
     <row r="74" spans="1:24">
-      <c r="A74" s="9" t="s">
+      <c r="A74" s="12" t="s">
         <v>79</v>
       </c>
-      <c r="B74" s="7"/>
+      <c r="B74" s="13"/>
       <c r="C74" s="2"/>
       <c r="D74" s="2">
         <v>210</v>
@@ -2936,10 +2949,10 @@
       <c r="X74" s="2"/>
     </row>
     <row r="75" spans="1:24">
-      <c r="A75" s="11" t="s">
+      <c r="A75" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="B75" s="7"/>
+      <c r="B75" s="13"/>
       <c r="C75" s="2"/>
       <c r="D75" s="2"/>
       <c r="E75" s="4">
@@ -2966,10 +2979,10 @@
       <c r="X75" s="2"/>
     </row>
     <row r="76" spans="1:24">
-      <c r="A76" s="9" t="s">
+      <c r="A76" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="B76" s="7"/>
+      <c r="B76" s="13"/>
       <c r="C76" s="2"/>
       <c r="D76" s="2"/>
       <c r="E76" s="4">
@@ -2996,10 +3009,10 @@
       <c r="X76" s="2"/>
     </row>
     <row r="77" spans="1:24">
-      <c r="A77" s="9" t="s">
+      <c r="A77" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="B77" s="7"/>
+      <c r="B77" s="13"/>
       <c r="C77" s="2"/>
       <c r="D77" s="2"/>
       <c r="E77" s="4">
@@ -3026,10 +3039,10 @@
       <c r="X77" s="2"/>
     </row>
     <row r="78" spans="1:24">
-      <c r="A78" s="9" t="s">
+      <c r="A78" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="B78" s="7"/>
+      <c r="B78" s="13"/>
       <c r="C78" s="2"/>
       <c r="D78" s="2"/>
       <c r="E78" s="4">
@@ -3056,7 +3069,7 @@
       <c r="X78" s="2"/>
     </row>
     <row r="79" spans="1:24">
-      <c r="A79" s="10" t="s">
+      <c r="A79" s="8" t="s">
         <v>84</v>
       </c>
       <c r="B79" s="7"/>
@@ -3065,7 +3078,7 @@
       <c r="E79" s="5">
         <v>6</v>
       </c>
-      <c r="F79" s="12" t="s">
+      <c r="F79" s="9" t="s">
         <v>85</v>
       </c>
       <c r="G79" s="7"/>
@@ -3088,7 +3101,7 @@
       <c r="X79" s="2"/>
     </row>
     <row r="80" spans="1:24">
-      <c r="A80" s="10" t="s">
+      <c r="A80" s="8" t="s">
         <v>86</v>
       </c>
       <c r="B80" s="7"/>
@@ -6421,89 +6434,90 @@
     </row>
   </sheetData>
   <mergeCells count="81">
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="A41:B41"/>
+    <mergeCell ref="A42:B42"/>
+    <mergeCell ref="A43:B43"/>
+    <mergeCell ref="A44:B44"/>
+    <mergeCell ref="A45:B45"/>
+    <mergeCell ref="A46:B46"/>
+    <mergeCell ref="A47:B47"/>
+    <mergeCell ref="A48:B48"/>
+    <mergeCell ref="A49:B49"/>
+    <mergeCell ref="A50:B50"/>
+    <mergeCell ref="A51:B51"/>
+    <mergeCell ref="A52:B52"/>
+    <mergeCell ref="A53:B53"/>
+    <mergeCell ref="A54:B54"/>
+    <mergeCell ref="A55:B55"/>
+    <mergeCell ref="A56:B56"/>
+    <mergeCell ref="A57:B57"/>
+    <mergeCell ref="A58:B58"/>
+    <mergeCell ref="A59:B59"/>
+    <mergeCell ref="A60:B60"/>
+    <mergeCell ref="A61:B61"/>
+    <mergeCell ref="A62:B62"/>
+    <mergeCell ref="A63:B63"/>
+    <mergeCell ref="A64:B64"/>
+    <mergeCell ref="A65:B65"/>
+    <mergeCell ref="A66:B66"/>
+    <mergeCell ref="A67:B67"/>
+    <mergeCell ref="A68:B68"/>
+    <mergeCell ref="A69:B69"/>
+    <mergeCell ref="A70:B70"/>
+    <mergeCell ref="A71:B71"/>
+    <mergeCell ref="A72:B72"/>
+    <mergeCell ref="A73:B73"/>
+    <mergeCell ref="A74:B74"/>
+    <mergeCell ref="A75:B75"/>
     <mergeCell ref="A76:B76"/>
     <mergeCell ref="A77:B77"/>
     <mergeCell ref="A78:B78"/>
     <mergeCell ref="A79:B79"/>
     <mergeCell ref="F79:G80"/>
     <mergeCell ref="A80:B80"/>
-    <mergeCell ref="A71:B71"/>
-    <mergeCell ref="A72:B72"/>
-    <mergeCell ref="A73:B73"/>
-    <mergeCell ref="A74:B74"/>
-    <mergeCell ref="A75:B75"/>
-    <mergeCell ref="A66:B66"/>
-    <mergeCell ref="A67:B67"/>
-    <mergeCell ref="A68:B68"/>
-    <mergeCell ref="A69:B69"/>
-    <mergeCell ref="A70:B70"/>
-    <mergeCell ref="A61:B61"/>
-    <mergeCell ref="A62:B62"/>
-    <mergeCell ref="A63:B63"/>
-    <mergeCell ref="A64:B64"/>
-    <mergeCell ref="A65:B65"/>
-    <mergeCell ref="A56:B56"/>
-    <mergeCell ref="A57:B57"/>
-    <mergeCell ref="A58:B58"/>
-    <mergeCell ref="A59:B59"/>
-    <mergeCell ref="A60:B60"/>
-    <mergeCell ref="A51:B51"/>
-    <mergeCell ref="A52:B52"/>
-    <mergeCell ref="A53:B53"/>
-    <mergeCell ref="A54:B54"/>
-    <mergeCell ref="A55:B55"/>
-    <mergeCell ref="A46:B46"/>
-    <mergeCell ref="A47:B47"/>
-    <mergeCell ref="A48:B48"/>
-    <mergeCell ref="A49:B49"/>
-    <mergeCell ref="A50:B50"/>
-    <mergeCell ref="A41:B41"/>
-    <mergeCell ref="A42:B42"/>
-    <mergeCell ref="A43:B43"/>
-    <mergeCell ref="A44:B44"/>
-    <mergeCell ref="A45:B45"/>
-    <mergeCell ref="A36:B36"/>
-    <mergeCell ref="A37:B37"/>
-    <mergeCell ref="A38:B38"/>
-    <mergeCell ref="A39:B39"/>
-    <mergeCell ref="A40:B40"/>
-    <mergeCell ref="A31:B31"/>
-    <mergeCell ref="A32:B32"/>
-    <mergeCell ref="A33:B33"/>
-    <mergeCell ref="A34:B34"/>
-    <mergeCell ref="A35:B35"/>
-    <mergeCell ref="A26:B26"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="A29:B29"/>
-    <mergeCell ref="A30:B30"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A5:B5"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update on 4.30 新增产品
</commit_message>
<xml_diff>
--- a/resources/4.30 新增产品.xlsx
+++ b/resources/4.30 新增产品.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hengchangqi/Documents/Singapore/Plan &amp; Note Internship/Part Time/WeChatProjects/TrinityGlobe/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA92537D-5A03-A84E-950C-5E77CB7F01AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37C45CC2-C336-2D45-AE64-975E03DDED86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="工作表1" sheetId="1" r:id="rId1"/>
@@ -363,7 +363,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -387,9 +387,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -673,7 +670,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="18" customHeight="1">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="7"/>
@@ -713,10 +710,10 @@
       <c r="X1" s="2"/>
     </row>
     <row r="2" spans="1:24" ht="18" customHeight="1">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="13"/>
+      <c r="B2" s="12"/>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
@@ -741,10 +738,10 @@
       <c r="X2" s="2"/>
     </row>
     <row r="3" spans="1:24" ht="18" customHeight="1">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="13"/>
+      <c r="B3" s="12"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2">
         <v>131</v>
@@ -773,10 +770,10 @@
       <c r="X3" s="2"/>
     </row>
     <row r="4" spans="1:24" ht="18" customHeight="1">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="13"/>
+      <c r="B4" s="12"/>
       <c r="C4" s="2"/>
       <c r="D4" s="2">
         <v>147</v>
@@ -805,10 +802,10 @@
       <c r="X4" s="2"/>
     </row>
     <row r="5" spans="1:24" ht="18" customHeight="1">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="13"/>
+      <c r="B5" s="12"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2">
         <v>240</v>
@@ -837,10 +834,10 @@
       <c r="X5" s="2"/>
     </row>
     <row r="6" spans="1:24" ht="18" customHeight="1">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="13"/>
+      <c r="B6" s="12"/>
       <c r="C6" s="2"/>
       <c r="D6" s="2">
         <v>448</v>
@@ -869,10 +866,10 @@
       <c r="X6" s="2"/>
     </row>
     <row r="7" spans="1:24" ht="18" customHeight="1">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="13"/>
+      <c r="B7" s="12"/>
       <c r="C7" s="2"/>
       <c r="D7" s="2">
         <v>540</v>
@@ -901,10 +898,10 @@
       <c r="X7" s="2"/>
     </row>
     <row r="8" spans="1:24" ht="18" customHeight="1">
-      <c r="A8" s="12" t="s">
+      <c r="A8" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="13"/>
+      <c r="B8" s="12"/>
       <c r="C8" s="2"/>
       <c r="D8" s="2">
         <v>2800</v>
@@ -933,10 +930,10 @@
       <c r="X8" s="2"/>
     </row>
     <row r="9" spans="1:24" ht="18" customHeight="1">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="13"/>
+      <c r="B9" s="12"/>
       <c r="C9" s="2"/>
       <c r="D9" s="2">
         <v>4690</v>
@@ -965,10 +962,10 @@
       <c r="X9" s="2"/>
     </row>
     <row r="10" spans="1:24" ht="18" customHeight="1">
-      <c r="A10" s="12" t="s">
+      <c r="A10" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="13"/>
+      <c r="B10" s="12"/>
       <c r="C10" s="2"/>
       <c r="D10" s="2">
         <v>6800</v>
@@ -997,7 +994,7 @@
       <c r="X10" s="2"/>
     </row>
     <row r="11" spans="1:24" ht="18" customHeight="1">
-      <c r="A11" s="10" t="s">
+      <c r="A11" s="9" t="s">
         <v>16</v>
       </c>
       <c r="B11" s="7"/>
@@ -1025,10 +1022,10 @@
       <c r="X11" s="2"/>
     </row>
     <row r="12" spans="1:24" ht="18" customHeight="1">
-      <c r="A12" s="12" t="s">
+      <c r="A12" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="13"/>
+      <c r="B12" s="12"/>
       <c r="C12" s="2">
         <v>129</v>
       </c>
@@ -1059,10 +1056,10 @@
       <c r="X12" s="2"/>
     </row>
     <row r="13" spans="1:24" ht="18" customHeight="1">
-      <c r="A13" s="12" t="s">
+      <c r="A13" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="B13" s="13"/>
+      <c r="B13" s="12"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2">
         <v>858</v>
@@ -1091,10 +1088,10 @@
       <c r="X13" s="2"/>
     </row>
     <row r="14" spans="1:24" ht="18" customHeight="1">
-      <c r="A14" s="12" t="s">
+      <c r="A14" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="B14" s="13"/>
+      <c r="B14" s="12"/>
       <c r="C14" s="2">
         <v>237</v>
       </c>
@@ -1125,10 +1122,10 @@
       <c r="X14" s="2"/>
     </row>
     <row r="15" spans="1:24" ht="18" customHeight="1">
-      <c r="A15" s="12" t="s">
+      <c r="A15" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="B15" s="13"/>
+      <c r="B15" s="12"/>
       <c r="C15" s="2"/>
       <c r="D15" s="2">
         <v>1038</v>
@@ -1157,7 +1154,7 @@
       <c r="X15" s="2"/>
     </row>
     <row r="16" spans="1:24" ht="18" customHeight="1">
-      <c r="A16" s="10" t="s">
+      <c r="A16" s="9" t="s">
         <v>21</v>
       </c>
       <c r="B16" s="7"/>
@@ -1185,10 +1182,10 @@
       <c r="X16" s="2"/>
     </row>
     <row r="17" spans="1:24" ht="18" customHeight="1">
-      <c r="A17" s="12" t="s">
+      <c r="A17" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="B17" s="13"/>
+      <c r="B17" s="12"/>
       <c r="C17" s="2"/>
       <c r="D17" s="2">
         <v>89</v>
@@ -1217,10 +1214,10 @@
       <c r="X17" s="2"/>
     </row>
     <row r="18" spans="1:24" ht="18" customHeight="1">
-      <c r="A18" s="12" t="s">
+      <c r="A18" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="B18" s="13"/>
+      <c r="B18" s="12"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2">
         <v>232</v>
@@ -1249,10 +1246,10 @@
       <c r="X18" s="2"/>
     </row>
     <row r="19" spans="1:24" ht="18" customHeight="1">
-      <c r="A19" s="12" t="s">
+      <c r="A19" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="B19" s="13"/>
+      <c r="B19" s="12"/>
       <c r="C19" s="2"/>
       <c r="D19" s="2">
         <v>1398</v>
@@ -1281,10 +1278,10 @@
       <c r="X19" s="2"/>
     </row>
     <row r="20" spans="1:24" ht="18" customHeight="1">
-      <c r="A20" s="12" t="s">
+      <c r="A20" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="B20" s="13"/>
+      <c r="B20" s="12"/>
       <c r="C20" s="2">
         <v>77</v>
       </c>
@@ -1315,10 +1312,10 @@
       <c r="X20" s="2"/>
     </row>
     <row r="21" spans="1:24" ht="18" customHeight="1">
-      <c r="A21" s="12" t="s">
+      <c r="A21" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="B21" s="13"/>
+      <c r="B21" s="12"/>
       <c r="C21" s="2">
         <v>200</v>
       </c>
@@ -1349,10 +1346,10 @@
       <c r="X21" s="2"/>
     </row>
     <row r="22" spans="1:24" ht="18" customHeight="1">
-      <c r="A22" s="12" t="s">
+      <c r="A22" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="B22" s="13"/>
+      <c r="B22" s="12"/>
       <c r="C22" s="5"/>
       <c r="D22" s="5"/>
       <c r="E22" s="5">
@@ -1379,10 +1376,10 @@
       <c r="X22" s="2"/>
     </row>
     <row r="23" spans="1:24" ht="18" customHeight="1">
-      <c r="A23" s="12" t="s">
+      <c r="A23" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="B23" s="13"/>
+      <c r="B23" s="12"/>
       <c r="C23" s="5"/>
       <c r="D23" s="5"/>
       <c r="E23" s="5">
@@ -1409,7 +1406,7 @@
       <c r="X23" s="2"/>
     </row>
     <row r="24" spans="1:24" ht="18" customHeight="1">
-      <c r="A24" s="10" t="s">
+      <c r="A24" s="9" t="s">
         <v>29</v>
       </c>
       <c r="B24" s="7"/>
@@ -1437,10 +1434,10 @@
       <c r="X24" s="2"/>
     </row>
     <row r="25" spans="1:24" ht="18" customHeight="1">
-      <c r="A25" s="12" t="s">
+      <c r="A25" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="B25" s="13"/>
+      <c r="B25" s="12"/>
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
       <c r="E25" s="2">
@@ -1467,10 +1464,10 @@
       <c r="X25" s="2"/>
     </row>
     <row r="26" spans="1:24" ht="18" customHeight="1">
-      <c r="A26" s="12" t="s">
+      <c r="A26" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="B26" s="13"/>
+      <c r="B26" s="12"/>
       <c r="C26" s="2"/>
       <c r="D26" s="2"/>
       <c r="E26" s="2">
@@ -1497,10 +1494,10 @@
       <c r="X26" s="2"/>
     </row>
     <row r="27" spans="1:24" ht="18" customHeight="1">
-      <c r="A27" s="12" t="s">
+      <c r="A27" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="B27" s="13"/>
+      <c r="B27" s="12"/>
       <c r="C27" s="2"/>
       <c r="D27" s="2"/>
       <c r="E27" s="2">
@@ -1527,10 +1524,10 @@
       <c r="X27" s="2"/>
     </row>
     <row r="28" spans="1:24" ht="18" customHeight="1">
-      <c r="A28" s="12" t="s">
+      <c r="A28" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="B28" s="13"/>
+      <c r="B28" s="12"/>
       <c r="C28" s="2"/>
       <c r="D28" s="2"/>
       <c r="E28" s="2">
@@ -1557,10 +1554,10 @@
       <c r="X28" s="2"/>
     </row>
     <row r="29" spans="1:24" ht="18" customHeight="1">
-      <c r="A29" s="12" t="s">
+      <c r="A29" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="B29" s="13"/>
+      <c r="B29" s="12"/>
       <c r="C29" s="2"/>
       <c r="D29" s="2"/>
       <c r="E29" s="2">
@@ -1587,10 +1584,10 @@
       <c r="X29" s="2"/>
     </row>
     <row r="30" spans="1:24" ht="18" customHeight="1">
-      <c r="A30" s="12" t="s">
+      <c r="A30" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="B30" s="13"/>
+      <c r="B30" s="12"/>
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
       <c r="E30" s="2">
@@ -1617,10 +1614,10 @@
       <c r="X30" s="2"/>
     </row>
     <row r="31" spans="1:24" ht="18" customHeight="1">
-      <c r="A31" s="12" t="s">
+      <c r="A31" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="B31" s="13"/>
+      <c r="B31" s="12"/>
       <c r="C31" s="2"/>
       <c r="D31" s="2"/>
       <c r="E31" s="2">
@@ -1647,10 +1644,10 @@
       <c r="X31" s="2"/>
     </row>
     <row r="32" spans="1:24" ht="18" customHeight="1">
-      <c r="A32" s="12" t="s">
+      <c r="A32" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="B32" s="13"/>
+      <c r="B32" s="12"/>
       <c r="C32" s="2"/>
       <c r="D32" s="2"/>
       <c r="E32" s="2">
@@ -1677,10 +1674,10 @@
       <c r="X32" s="2"/>
     </row>
     <row r="33" spans="1:24" ht="18" customHeight="1">
-      <c r="A33" s="12" t="s">
+      <c r="A33" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="B33" s="13"/>
+      <c r="B33" s="12"/>
       <c r="C33" s="2"/>
       <c r="D33" s="2"/>
       <c r="E33" s="2">
@@ -1707,10 +1704,10 @@
       <c r="X33" s="2"/>
     </row>
     <row r="34" spans="1:24" ht="18" customHeight="1">
-      <c r="A34" s="12" t="s">
+      <c r="A34" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="B34" s="13"/>
+      <c r="B34" s="12"/>
       <c r="C34" s="2"/>
       <c r="D34" s="2"/>
       <c r="E34" s="2">
@@ -1737,10 +1734,10 @@
       <c r="X34" s="2"/>
     </row>
     <row r="35" spans="1:24" ht="18" customHeight="1">
-      <c r="A35" s="12" t="s">
+      <c r="A35" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="B35" s="13"/>
+      <c r="B35" s="12"/>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
       <c r="E35" s="2">
@@ -1767,10 +1764,10 @@
       <c r="X35" s="2"/>
     </row>
     <row r="36" spans="1:24" ht="18" customHeight="1">
-      <c r="A36" s="12" t="s">
+      <c r="A36" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="B36" s="13"/>
+      <c r="B36" s="12"/>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
       <c r="E36" s="2">
@@ -1797,10 +1794,10 @@
       <c r="X36" s="2"/>
     </row>
     <row r="37" spans="1:24" ht="18" customHeight="1">
-      <c r="A37" s="12" t="s">
+      <c r="A37" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="B37" s="13"/>
+      <c r="B37" s="12"/>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>
       <c r="E37" s="2">
@@ -1827,7 +1824,7 @@
       <c r="X37" s="2"/>
     </row>
     <row r="38" spans="1:24" ht="18" customHeight="1">
-      <c r="A38" s="10" t="s">
+      <c r="A38" s="9" t="s">
         <v>43</v>
       </c>
       <c r="B38" s="7"/>
@@ -1855,10 +1852,10 @@
       <c r="X38" s="2"/>
     </row>
     <row r="39" spans="1:24" ht="18" customHeight="1">
-      <c r="A39" s="12" t="s">
+      <c r="A39" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="B39" s="13"/>
+      <c r="B39" s="12"/>
       <c r="C39" s="2"/>
       <c r="D39" s="2"/>
       <c r="E39" s="2">
@@ -1885,10 +1882,10 @@
       <c r="X39" s="2"/>
     </row>
     <row r="40" spans="1:24" ht="18" customHeight="1">
-      <c r="A40" s="12" t="s">
+      <c r="A40" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="B40" s="13"/>
+      <c r="B40" s="12"/>
       <c r="C40" s="2"/>
       <c r="D40" s="2"/>
       <c r="E40" s="2">
@@ -2035,10 +2032,10 @@
       <c r="X44" s="2"/>
     </row>
     <row r="45" spans="1:24">
-      <c r="A45" s="12" t="s">
+      <c r="A45" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="B45" s="13"/>
+      <c r="B45" s="12"/>
       <c r="C45" s="2"/>
       <c r="D45" s="2"/>
       <c r="E45" s="2">
@@ -2065,10 +2062,10 @@
       <c r="X45" s="2"/>
     </row>
     <row r="46" spans="1:24">
-      <c r="A46" s="12" t="s">
+      <c r="A46" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="B46" s="13"/>
+      <c r="B46" s="12"/>
       <c r="C46" s="2"/>
       <c r="D46" s="2"/>
       <c r="E46" s="2">
@@ -2095,10 +2092,10 @@
       <c r="X46" s="2"/>
     </row>
     <row r="47" spans="1:24">
-      <c r="A47" s="12" t="s">
+      <c r="A47" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="B47" s="13"/>
+      <c r="B47" s="12"/>
       <c r="C47" s="2"/>
       <c r="D47" s="2"/>
       <c r="E47" s="2">
@@ -2125,10 +2122,10 @@
       <c r="X47" s="2"/>
     </row>
     <row r="48" spans="1:24">
-      <c r="A48" s="12" t="s">
+      <c r="A48" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="B48" s="13"/>
+      <c r="B48" s="12"/>
       <c r="C48" s="2"/>
       <c r="D48" s="2"/>
       <c r="E48" s="2">
@@ -2155,10 +2152,10 @@
       <c r="X48" s="2"/>
     </row>
     <row r="49" spans="1:24">
-      <c r="A49" s="12" t="s">
+      <c r="A49" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="B49" s="13"/>
+      <c r="B49" s="12"/>
       <c r="C49" s="2"/>
       <c r="D49" s="2"/>
       <c r="E49" s="2">
@@ -2185,10 +2182,10 @@
       <c r="X49" s="2"/>
     </row>
     <row r="50" spans="1:24">
-      <c r="A50" s="12" t="s">
+      <c r="A50" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="B50" s="13"/>
+      <c r="B50" s="12"/>
       <c r="C50" s="2"/>
       <c r="D50" s="2"/>
       <c r="E50" s="2">
@@ -2215,10 +2212,10 @@
       <c r="X50" s="2"/>
     </row>
     <row r="51" spans="1:24">
-      <c r="A51" s="12" t="s">
+      <c r="A51" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="B51" s="13"/>
+      <c r="B51" s="12"/>
       <c r="C51" s="2"/>
       <c r="D51" s="2"/>
       <c r="E51" s="2">
@@ -2245,10 +2242,10 @@
       <c r="X51" s="2"/>
     </row>
     <row r="52" spans="1:24">
-      <c r="A52" s="12" t="s">
+      <c r="A52" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="B52" s="13"/>
+      <c r="B52" s="12"/>
       <c r="C52" s="2"/>
       <c r="D52" s="2"/>
       <c r="E52" s="2">
@@ -2275,7 +2272,7 @@
       <c r="X52" s="2"/>
     </row>
     <row r="53" spans="1:24">
-      <c r="A53" s="10" t="s">
+      <c r="A53" s="9" t="s">
         <v>58</v>
       </c>
       <c r="B53" s="7"/>
@@ -2303,10 +2300,10 @@
       <c r="X53" s="2"/>
     </row>
     <row r="54" spans="1:24">
-      <c r="A54" s="12" t="s">
+      <c r="A54" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="B54" s="13"/>
+      <c r="B54" s="12"/>
       <c r="C54" s="2"/>
       <c r="D54" s="2"/>
       <c r="E54" s="2">
@@ -2333,10 +2330,10 @@
       <c r="X54" s="2"/>
     </row>
     <row r="55" spans="1:24">
-      <c r="A55" s="12" t="s">
+      <c r="A55" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="B55" s="13"/>
+      <c r="B55" s="12"/>
       <c r="C55" s="2"/>
       <c r="D55" s="2"/>
       <c r="E55" s="2">
@@ -2363,10 +2360,10 @@
       <c r="X55" s="2"/>
     </row>
     <row r="56" spans="1:24">
-      <c r="A56" s="12" t="s">
+      <c r="A56" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="B56" s="13"/>
+      <c r="B56" s="12"/>
       <c r="C56" s="2"/>
       <c r="D56" s="2"/>
       <c r="E56" s="2">
@@ -2393,10 +2390,10 @@
       <c r="X56" s="2"/>
     </row>
     <row r="57" spans="1:24">
-      <c r="A57" s="12" t="s">
+      <c r="A57" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="B57" s="13"/>
+      <c r="B57" s="12"/>
       <c r="C57" s="2"/>
       <c r="D57" s="2"/>
       <c r="E57" s="2">
@@ -2423,10 +2420,10 @@
       <c r="X57" s="2"/>
     </row>
     <row r="58" spans="1:24">
-      <c r="A58" s="12" t="s">
+      <c r="A58" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="B58" s="13"/>
+      <c r="B58" s="12"/>
       <c r="C58" s="2"/>
       <c r="D58" s="2">
         <v>228</v>
@@ -2455,10 +2452,10 @@
       <c r="X58" s="2"/>
     </row>
     <row r="59" spans="1:24">
-      <c r="A59" s="12" t="s">
+      <c r="A59" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="B59" s="13"/>
+      <c r="B59" s="12"/>
       <c r="C59" s="2"/>
       <c r="D59" s="2">
         <v>340</v>
@@ -2487,10 +2484,10 @@
       <c r="X59" s="2"/>
     </row>
     <row r="60" spans="1:24">
-      <c r="A60" s="12" t="s">
+      <c r="A60" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="B60" s="13"/>
+      <c r="B60" s="12"/>
       <c r="C60" s="2"/>
       <c r="D60" s="2"/>
       <c r="E60" s="4">
@@ -2517,10 +2514,10 @@
       <c r="X60" s="2"/>
     </row>
     <row r="61" spans="1:24">
-      <c r="A61" s="12" t="s">
+      <c r="A61" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B61" s="13"/>
+      <c r="B61" s="12"/>
       <c r="C61" s="2"/>
       <c r="D61" s="2"/>
       <c r="E61" s="4">
@@ -2547,10 +2544,10 @@
       <c r="X61" s="2"/>
     </row>
     <row r="62" spans="1:24">
-      <c r="A62" s="12" t="s">
+      <c r="A62" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="B62" s="13"/>
+      <c r="B62" s="12"/>
       <c r="C62" s="2"/>
       <c r="D62" s="2"/>
       <c r="E62" s="4">
@@ -2577,10 +2574,10 @@
       <c r="X62" s="2"/>
     </row>
     <row r="63" spans="1:24">
-      <c r="A63" s="12" t="s">
+      <c r="A63" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="B63" s="13"/>
+      <c r="B63" s="12"/>
       <c r="C63" s="2"/>
       <c r="D63" s="2"/>
       <c r="E63" s="4">
@@ -2607,7 +2604,7 @@
       <c r="X63" s="2"/>
     </row>
     <row r="64" spans="1:24">
-      <c r="A64" s="10" t="s">
+      <c r="A64" s="9" t="s">
         <v>69</v>
       </c>
       <c r="B64" s="7"/>
@@ -2635,10 +2632,10 @@
       <c r="X64" s="2"/>
     </row>
     <row r="65" spans="1:24">
-      <c r="A65" s="12" t="s">
+      <c r="A65" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="B65" s="13"/>
+      <c r="B65" s="12"/>
       <c r="C65" s="2"/>
       <c r="D65" s="2">
         <v>324</v>
@@ -2667,10 +2664,10 @@
       <c r="X65" s="2"/>
     </row>
     <row r="66" spans="1:24">
-      <c r="A66" s="12" t="s">
+      <c r="A66" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="B66" s="13"/>
+      <c r="B66" s="12"/>
       <c r="C66" s="2"/>
       <c r="D66" s="2">
         <v>263</v>
@@ -2699,10 +2696,10 @@
       <c r="X66" s="2"/>
     </row>
     <row r="67" spans="1:24">
-      <c r="A67" s="12" t="s">
+      <c r="A67" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="B67" s="13"/>
+      <c r="B67" s="12"/>
       <c r="C67" s="2"/>
       <c r="D67" s="2">
         <v>496</v>
@@ -2731,10 +2728,10 @@
       <c r="X67" s="2"/>
     </row>
     <row r="68" spans="1:24">
-      <c r="A68" s="12" t="s">
+      <c r="A68" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="B68" s="13"/>
+      <c r="B68" s="12"/>
       <c r="C68" s="2"/>
       <c r="D68" s="2">
         <v>88</v>
@@ -2763,10 +2760,10 @@
       <c r="X68" s="2"/>
     </row>
     <row r="69" spans="1:24">
-      <c r="A69" s="12" t="s">
+      <c r="A69" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="B69" s="13"/>
+      <c r="B69" s="12"/>
       <c r="C69" s="2"/>
       <c r="D69" s="2">
         <v>116</v>
@@ -2795,10 +2792,10 @@
       <c r="X69" s="2"/>
     </row>
     <row r="70" spans="1:24">
-      <c r="A70" s="12" t="s">
+      <c r="A70" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="B70" s="13"/>
+      <c r="B70" s="12"/>
       <c r="C70" s="2"/>
       <c r="D70" s="2">
         <v>124</v>
@@ -2827,10 +2824,10 @@
       <c r="X70" s="2"/>
     </row>
     <row r="71" spans="1:24">
-      <c r="A71" s="12" t="s">
+      <c r="A71" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="B71" s="13"/>
+      <c r="B71" s="12"/>
       <c r="C71" s="5"/>
       <c r="D71" s="5"/>
       <c r="E71" s="5">
@@ -2857,10 +2854,10 @@
       <c r="X71" s="2"/>
     </row>
     <row r="72" spans="1:24">
-      <c r="A72" s="12" t="s">
+      <c r="A72" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="B72" s="13"/>
+      <c r="B72" s="12"/>
       <c r="C72" s="5"/>
       <c r="D72" s="5"/>
       <c r="E72" s="5">
@@ -2887,10 +2884,10 @@
       <c r="X72" s="2"/>
     </row>
     <row r="73" spans="1:24">
-      <c r="A73" s="12" t="s">
+      <c r="A73" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="B73" s="13"/>
+      <c r="B73" s="12"/>
       <c r="C73" s="5"/>
       <c r="D73" s="5"/>
       <c r="E73" s="5">
@@ -2917,10 +2914,10 @@
       <c r="X73" s="2"/>
     </row>
     <row r="74" spans="1:24">
-      <c r="A74" s="12" t="s">
+      <c r="A74" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="B74" s="13"/>
+      <c r="B74" s="12"/>
       <c r="C74" s="2"/>
       <c r="D74" s="2">
         <v>210</v>
@@ -2949,10 +2946,10 @@
       <c r="X74" s="2"/>
     </row>
     <row r="75" spans="1:24">
-      <c r="A75" s="14" t="s">
+      <c r="A75" s="13" t="s">
         <v>80</v>
       </c>
-      <c r="B75" s="13"/>
+      <c r="B75" s="12"/>
       <c r="C75" s="2"/>
       <c r="D75" s="2"/>
       <c r="E75" s="4">
@@ -2979,10 +2976,10 @@
       <c r="X75" s="2"/>
     </row>
     <row r="76" spans="1:24">
-      <c r="A76" s="12" t="s">
+      <c r="A76" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="B76" s="13"/>
+      <c r="B76" s="12"/>
       <c r="C76" s="2"/>
       <c r="D76" s="2"/>
       <c r="E76" s="4">
@@ -3009,10 +3006,10 @@
       <c r="X76" s="2"/>
     </row>
     <row r="77" spans="1:24">
-      <c r="A77" s="12" t="s">
+      <c r="A77" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="B77" s="13"/>
+      <c r="B77" s="12"/>
       <c r="C77" s="2"/>
       <c r="D77" s="2"/>
       <c r="E77" s="4">
@@ -3039,10 +3036,10 @@
       <c r="X77" s="2"/>
     </row>
     <row r="78" spans="1:24">
-      <c r="A78" s="12" t="s">
+      <c r="A78" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="B78" s="13"/>
+      <c r="B78" s="12"/>
       <c r="C78" s="2"/>
       <c r="D78" s="2"/>
       <c r="E78" s="4">
@@ -3069,16 +3066,16 @@
       <c r="X78" s="2"/>
     </row>
     <row r="79" spans="1:24">
-      <c r="A79" s="8" t="s">
+      <c r="A79" s="11" t="s">
         <v>84</v>
       </c>
-      <c r="B79" s="7"/>
+      <c r="B79" s="12"/>
       <c r="C79" s="5"/>
       <c r="D79" s="5"/>
       <c r="E79" s="5">
         <v>6</v>
       </c>
-      <c r="F79" s="9" t="s">
+      <c r="F79" s="8" t="s">
         <v>85</v>
       </c>
       <c r="G79" s="7"/>
@@ -3101,10 +3098,10 @@
       <c r="X79" s="2"/>
     </row>
     <row r="80" spans="1:24">
-      <c r="A80" s="8" t="s">
+      <c r="A80" s="11" t="s">
         <v>86</v>
       </c>
-      <c r="B80" s="7"/>
+      <c r="B80" s="12"/>
       <c r="C80" s="5"/>
       <c r="D80" s="5"/>
       <c r="E80" s="5">

</xml_diff>